<commit_message>
Refactor automation framework and clean repository~
</commit_message>
<xml_diff>
--- a/testData/Open_cart_Login_credentials.xlsx
+++ b/testData/Open_cart_Login_credentials.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5C5283F7-F0AC-4F91-A29F-A56104D6C861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{7D4C92D9-8884-4DC8-9F4A-8F9FA8FD620E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{28D2D463-07ED-4AE7-9A21-E79917FE6FFE}"/>
   </bookViews>
@@ -16,21 +16,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
   <si>
     <t>username</t>
   </si>
@@ -56,22 +47,22 @@
     <t>Aa@123456</t>
   </si>
   <si>
-    <t>azwewed@gmail.com</t>
-  </si>
-  <si>
     <t>Invalid</t>
   </si>
   <si>
-    <t>werrwefw@gmail.com</t>
-  </si>
-  <si>
-    <t>23@321</t>
-  </si>
-  <si>
-    <t>asfqwfasf@gmail.com</t>
-  </si>
-  <si>
-    <t>aefwfd</t>
+    <t>weefdfw@gmail.com</t>
+  </si>
+  <si>
+    <t>eefae@weefdsf</t>
+  </si>
+  <si>
+    <t>swerwe@gmail.com</t>
+  </si>
+  <si>
+    <t>werdwerwer</t>
+  </si>
+  <si>
+    <t>azeez@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -126,10 +117,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -484,47 +473,47 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="3">
-        <v>3243232</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>9</v>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -540,14 +529,15 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{B5CB43C4-5C29-4238-9947-EA430EA88807}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{5DCDE9B2-FBC0-4F9C-822D-C682AE746FDC}"/>
-    <hyperlink ref="A6" r:id="rId3" xr:uid="{1B1C49D9-8F7A-41D0-AD34-F225E5A9D87D}"/>
-    <hyperlink ref="B6" r:id="rId4" xr:uid="{DCE7F366-965F-48BF-9623-EAC1F404BA19}"/>
-    <hyperlink ref="A3" r:id="rId5" xr:uid="{C1E4D7AE-3CA4-4627-AE48-AFB59940D129}"/>
-    <hyperlink ref="A4" r:id="rId6" xr:uid="{B4396B96-FB60-4A03-979B-EE8D6D82935D}"/>
-    <hyperlink ref="B4" r:id="rId7" xr:uid="{5D49E919-502F-4A77-A425-020F5B4C2253}"/>
-    <hyperlink ref="A5" r:id="rId8" xr:uid="{8610371C-E957-415A-A679-D9FFBCE2A3D6}"/>
+    <hyperlink ref="A6" r:id="rId1" xr:uid="{DC0ED607-ACC3-475F-9C79-C673A83BFE22}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{C96BD277-3013-4F3E-8AEB-FC62B726A536}"/>
+    <hyperlink ref="A2" r:id="rId3" xr:uid="{B5CB43C4-5C29-4238-9947-EA430EA88807}"/>
+    <hyperlink ref="B2" r:id="rId4" xr:uid="{5DCDE9B2-FBC0-4F9C-822D-C682AE746FDC}"/>
+    <hyperlink ref="A5" r:id="rId5" xr:uid="{DC0ED607-ACC3-475F-9C79-C673A83BFE22}"/>
+    <hyperlink ref="B5" r:id="rId6" xr:uid="{C96BD277-3013-4F3E-8AEB-FC62B726A536}"/>
+    <hyperlink ref="A4" r:id="rId7" xr:uid="{0C4FD4FF-E0ED-44A9-8175-5C5415A5BC1B}"/>
+    <hyperlink ref="A3" r:id="rId8" xr:uid="{8B93796A-E593-4A65-80AA-B0CF4BA6D5EE}"/>
+    <hyperlink ref="B3" r:id="rId9" xr:uid="{69ABEB79-3B7B-4743-B913-16199EC8D48C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>